<commit_message>
Updated training data with fixed codes in quotation manager and entered "Jane Doe" as an alias
</commit_message>
<xml_diff>
--- a/Training Data - Code Manager.xlsx
+++ b/Training Data - Code Manager.xlsx
@@ -1,22 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11011"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aarhusuniversitet-my.sharepoint.com/personal/au687587_uni_au_dk/Documents/Data/Althea/althea/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_5159A21C65F1497C83ABE444F6A6E78A4FAEB8BF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D032C6DD-869D-EB4D-BA7E-327732B78208}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="120" windowWidth="14940" windowHeight="9225" activeTab="0"/>
+    <workbookView xWindow="30240" yWindow="-3840" windowWidth="51200" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId3"/>
-    <sheet name="Info" sheetId="2" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Info" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="29">
   <si>
     <r>
       <rPr>
@@ -212,13 +217,16 @@
       </rPr>
       <t>Date:</t>
     </r>
+  </si>
+  <si>
+    <t>Jane Doe</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="4">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color theme="1"/>
@@ -227,12 +235,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -260,168 +262,38 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
-      <alignment/>
-      <protection/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="8">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-  </cellStyleXfs>
-  <cellXfs count="16">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
-      <protection/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
-      <protection/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
-      <protection/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" wrapText="1"/>
-      <protection/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
-      <protection/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection/>
-    </xf>
-    <xf numFmtId="15" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
-      <protection/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
-      <protection/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" wrapText="1"/>
-      <protection/>
-    </xf>
-    <xf numFmtId="15" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection/>
     </xf>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="15" builtinId="5"/>
-    <cellStyle name="Currency" xfId="16" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="17" builtinId="7"/>
-    <cellStyle name="Comma" xfId="18" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="19" builtinId="6"/>
   </cellStyles>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -729,350 +601,350 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{d8f61514-5d2e-40a7-8f1b-98b0cb3cbdb0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8F61514-5D2E-40A7-8F1B-98B0CB3CBDB0}">
   <dimension ref="A1:J11"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="24.714285714285715" customWidth="1"/>
-    <col min="2" max="2" width="16.428571428571427" customWidth="1"/>
-    <col min="3" max="4" width="8.857142857142858" customWidth="1"/>
+    <col min="1" max="1" width="24.6640625" customWidth="1"/>
+    <col min="2" max="2" width="16.5" customWidth="1"/>
+    <col min="3" max="4" width="8.83203125" customWidth="1"/>
     <col min="5" max="5" width="20" customWidth="1"/>
-    <col min="6" max="6" width="20.714285714285715" customWidth="1"/>
-    <col min="7" max="7" width="17.142857142857142" customWidth="1"/>
-    <col min="8" max="8" width="15.285714285714286" customWidth="1"/>
-    <col min="9" max="9" width="17.142857142857142" customWidth="1"/>
+    <col min="6" max="6" width="20.6640625" customWidth="1"/>
+    <col min="7" max="7" width="17.1640625" customWidth="1"/>
+    <col min="8" max="8" width="15.33203125" customWidth="1"/>
+    <col min="9" max="9" width="17.1640625" customWidth="1"/>
     <col min="10" max="10" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:10" ht="15" x14ac:dyDescent="0.15">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="14.25">
-      <c r="A2" s="6" t="s">
+    <row r="2" spans="1:10" ht="15" x14ac:dyDescent="0.15">
+      <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="9">
+      <c r="B2" s="3">
         <v>23</v>
       </c>
-      <c r="C2" s="9">
+      <c r="C2" s="3">
         <v>0</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="9">
+      <c r="E2" s="3">
         <v>1</v>
       </c>
-      <c r="F2" s="10"/>
-      <c r="G2" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="H2" s="12">
+      <c r="F2" s="4"/>
+      <c r="G2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H2" s="5">
         <v>46247.564363425925</v>
       </c>
-      <c r="I2" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="J2" s="12">
+      <c r="I2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="J2" s="5">
         <v>46247.564363425925</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="14.25">
-      <c r="A3" s="6" t="s">
+    <row r="3" spans="1:10" ht="15" x14ac:dyDescent="0.15">
+      <c r="A3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="3">
         <v>15</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="3">
         <v>0</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="9">
+      <c r="E3" s="3">
         <v>1</v>
       </c>
-      <c r="F3" s="10"/>
-      <c r="G3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="H3" s="12">
+      <c r="F3" s="4"/>
+      <c r="G3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H3" s="5">
         <v>46247.66265046296</v>
       </c>
-      <c r="I3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="J3" s="12">
+      <c r="I3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="J3" s="5">
         <v>46247.66265046296</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="14.25">
-      <c r="A4" s="6" t="s">
+    <row r="4" spans="1:10" ht="15" x14ac:dyDescent="0.15">
+      <c r="A4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="3">
         <v>16</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="3">
         <v>0</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="9">
+      <c r="E4" s="3">
         <v>1</v>
       </c>
-      <c r="F4" s="10"/>
-      <c r="G4" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="H4" s="12">
+      <c r="F4" s="4"/>
+      <c r="G4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H4" s="5">
         <v>46247.564363425925</v>
       </c>
-      <c r="I4" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="J4" s="12">
+      <c r="I4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="J4" s="5">
         <v>46247.564363425925</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="14.25">
-      <c r="A5" s="6" t="s">
+    <row r="5" spans="1:10" ht="15" x14ac:dyDescent="0.15">
+      <c r="A5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="9">
+      <c r="B5" s="3">
         <v>27</v>
       </c>
-      <c r="C5" s="9">
+      <c r="C5" s="3">
         <v>0</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="9">
+      <c r="E5" s="3">
         <v>1</v>
       </c>
-      <c r="F5" s="10"/>
-      <c r="G5" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="H5" s="12">
+      <c r="F5" s="4"/>
+      <c r="G5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H5" s="5">
         <v>46247.560752314814</v>
       </c>
-      <c r="I5" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="J5" s="12">
+      <c r="I5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="J5" s="5">
         <v>46247.560752314814</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="14.25">
-      <c r="A6" s="6" t="s">
+    <row r="6" spans="1:10" ht="15" x14ac:dyDescent="0.15">
+      <c r="A6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="3">
         <v>18</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="3">
         <v>0</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="9">
+      <c r="E6" s="3">
         <v>1</v>
       </c>
-      <c r="F6" s="10"/>
-      <c r="G6" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="H6" s="12">
+      <c r="F6" s="4"/>
+      <c r="G6" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H6" s="5">
         <v>46247.657210648147</v>
       </c>
-      <c r="I6" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="J6" s="12">
+      <c r="I6" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="J6" s="5">
         <v>46247.657210648147</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="14.25">
-      <c r="A7" s="6" t="s">
+    <row r="7" spans="1:10" ht="15" x14ac:dyDescent="0.15">
+      <c r="A7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="9">
+      <c r="B7" s="3">
         <v>27</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="3">
         <v>0</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="9">
+      <c r="E7" s="3">
         <v>1</v>
       </c>
-      <c r="F7" s="10"/>
-      <c r="G7" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="H7" s="12">
+      <c r="F7" s="4"/>
+      <c r="G7" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H7" s="5">
         <v>46247.565254629626</v>
       </c>
-      <c r="I7" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="J7" s="12">
+      <c r="I7" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="J7" s="5">
         <v>46247.565254629626</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="14.25">
-      <c r="A8" s="6" t="s">
+    <row r="8" spans="1:10" ht="15" x14ac:dyDescent="0.15">
+      <c r="A8" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="9">
+      <c r="B8" s="3">
         <v>11</v>
       </c>
-      <c r="C8" s="9">
+      <c r="C8" s="3">
         <v>0</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E8" s="9">
+      <c r="E8" s="3">
         <v>1</v>
       </c>
-      <c r="F8" s="10"/>
-      <c r="G8" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="H8" s="12">
+      <c r="F8" s="4"/>
+      <c r="G8" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H8" s="5">
         <v>46247.560752314814</v>
       </c>
-      <c r="I8" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="J8" s="12">
+      <c r="I8" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="J8" s="5">
         <v>46247.560752314814</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="14.25">
-      <c r="A9" s="6" t="s">
+    <row r="9" spans="1:10" ht="15" x14ac:dyDescent="0.15">
+      <c r="A9" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B9" s="9">
+      <c r="B9" s="3">
         <v>13</v>
       </c>
-      <c r="C9" s="9">
+      <c r="C9" s="3">
         <v>0</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="9">
+      <c r="E9" s="3">
         <v>1</v>
       </c>
-      <c r="F9" s="10"/>
-      <c r="G9" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="H9" s="12">
+      <c r="F9" s="4"/>
+      <c r="G9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H9" s="5">
         <v>46247.664340277777</v>
       </c>
-      <c r="I9" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="J9" s="12">
+      <c r="I9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="J9" s="5">
         <v>46247.664340277777</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="14.25">
-      <c r="A10" s="6" t="s">
+    <row r="10" spans="1:10" ht="15" x14ac:dyDescent="0.15">
+      <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="9">
+      <c r="B10" s="3">
         <v>15</v>
       </c>
-      <c r="C10" s="9">
+      <c r="C10" s="3">
         <v>0</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E10" s="9">
+      <c r="E10" s="3">
         <v>1</v>
       </c>
-      <c r="F10" s="10"/>
-      <c r="G10" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="H10" s="12">
+      <c r="F10" s="4"/>
+      <c r="G10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H10" s="5">
         <v>46247.564363425925</v>
       </c>
-      <c r="I10" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="J10" s="12">
+      <c r="I10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="J10" s="5">
         <v>46247.564363425925</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="14.25">
-      <c r="A11" s="6" t="s">
+    <row r="11" spans="1:10" ht="15" x14ac:dyDescent="0.15">
+      <c r="A11" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="9">
-        <v>28</v>
-      </c>
-      <c r="C11" s="9">
+      <c r="B11" s="3">
+        <v>28</v>
+      </c>
+      <c r="C11" s="3">
         <v>0</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E11" s="9">
+      <c r="E11" s="3">
         <v>1</v>
       </c>
-      <c r="F11" s="10"/>
-      <c r="G11" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="H11" s="12">
+      <c r="F11" s="4"/>
+      <c r="G11" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H11" s="5">
         <v>46247.669363425928</v>
       </c>
-      <c r="I11" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="J11" s="12">
+      <c r="I11" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="J11" s="5">
         <v>46247.669363425928</v>
       </c>
     </row>
@@ -1082,43 +954,43 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7588b0a6-fdf3-4ac5-b1c5-8cc7accfe0f8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7588B0A6-FDF3-4AC5-B1C5-8CC7ACCFE0F8}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="9.142857142857142" customWidth="1"/>
-    <col min="2" max="2" width="21.428571428571427" customWidth="1"/>
+    <col min="1" max="1" width="9.1640625" customWidth="1"/>
+    <col min="2" max="2" width="21.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:2" ht="15" x14ac:dyDescent="0.15">
+      <c r="A1" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="6" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15">
-      <c r="A2" s="13" t="s">
+    <row r="2" spans="1:2" ht="15" x14ac:dyDescent="0.15">
+      <c r="A2" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="6" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15">
-      <c r="A3" s="13" t="s">
+    <row r="3" spans="1:2" ht="15" x14ac:dyDescent="0.15">
+      <c r="A3" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="15">
-      <c r="A4" s="13" t="s">
+    <row r="4" spans="1:2" ht="15" x14ac:dyDescent="0.15">
+      <c r="A4" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="15">
+      <c r="B4" s="7">
         <v>46304.628541666665</v>
       </c>
     </row>

</xml_diff>